<commit_message>
bug_register: drop fixed rows; add B2/B3 for date i18n + export typing
User feedback: the register is an active worklist — fix history lives
in git, not here. Removed the 8 'Fixed' rows seeded earlier (B1-B8 of
the previous version) and renumbered the open items.

New open items:
  B1 — UI Polish (was B9; carried over).
  B2 — Dates not formatted per territory (screen + exports).
  B3 — Excel/PDF exports write cells as text instead of typed
       float/datetime, so Excel can't SUM or filter properly.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bug_register.xlsx
+++ b/docs/bug_register.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +37,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00635BFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCFFE4"/>
       </patternFill>
     </fill>
     <fill>
@@ -86,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -94,13 +89,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -468,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -484,10 +473,10 @@
     <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="56" customHeight="1">
+    <row r="1" ht="64" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AccGenie bug register. New bugs: append a row, give it the next B-id, default Status=Open (the row will go red); on fix, set Status=Fixed (the Status cell will go green) plus the version and commit short-hash. Severity: Critical=data loss / can't ship; High=blocks a flow; Medium=workaround exists; Low=cosmetic. Pending work / features live in pending_work.xlsx instead -- this file is defects only.</t>
+          <t>AccGenie bug register -- ACTIVE list only. Fixed bugs are removed (history lives in git). New bugs: append a row with the next B-id, Status=Open (the row goes red). When you ship a fix, delete the row rather than marking Fixed. Severity: Critical=data loss / can't ship; High=blocks a flow; Medium=workaround exists; Low=cosmetic. Pending features live in pending_work.xlsx -- this file is defects only.</t>
         </is>
       </c>
     </row>
@@ -566,42 +555,34 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Bank Reconciliation</t>
+          <t>UI Polish</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>auto_match greedy on (date, amount, sign) ties — arbitrarily paired same-day same-amount transactions, polluting reconciliations the user then had to manually unmatch.</t>
+          <t>Buttons too large or too small on multiple screens; some button text not visible (contrast / clipping); 'looks ugly on many screens'.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Two Rs.500 receipts on the same day -&gt; one bound to the wrong stmt line.</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>1.0.11</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>f3e433d</t>
-        </is>
-      </c>
+          <t>User-reported general impression. Specific screens not yet enumerated.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Now skips ambiguous buckets; ambiguous_skipped count surfaced in result.</t>
+          <t>Need user to list the specific screens. Cross-cuts pending_work.xlsx C1.</t>
         </is>
       </c>
     </row>
@@ -623,42 +604,34 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Bank Reconciliation</t>
+          <t>i18n -- Dates</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Split match dialog showed empty candidate list when bundled book legs had already been auto-matched 1-to-1 against unrelated stmt lines (same root cause as B1).</t>
+          <t>Dates are not formatted per territory on screen OR in exports. Whatever fixed format Qt/Python emits (typically yyyy-MM-dd or default locale) is used everywhere; non-Indian markets expect their own conventions (e.g. MM/DD/YYYY for US, DD/MM/YYYY for IN/EU).</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Click Split match on a settlement bank line -- dialog says 'no candidates' even though the legs exist in the period.</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>1.0.11</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>f3e433d</t>
-        </is>
-      </c>
+          <t>Open any report or the Day Book -- the Date column uses one hard-coded format regardless of company locale.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Resolved upstream by B1. Also added 'Undo all auto-matches' button.</t>
+          <t>Add a format_date() helper alongside core/i18n.py's format_currency. Wire it through display sites + exporters. See related B3 for export typing.</t>
         </is>
       </c>
     </row>
@@ -685,376 +658,34 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>All tables</t>
+          <t>Exports (Excel/PDF)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Click-to-sort headers did not work on any QTableWidget across 9 pages (Day Book, Bank Reco x4, Reports, Document Reader, Ledger Reco, Period Locks, Migration, Backup).</t>
+          <t>Excel/PDF exports write every cell as TEXT instead of using the column's real type. Amount cells become '"Rs. 1,234.56"' strings (no sum formula), date cells become '"19-May-2026"' strings (no sort/filter as date), counts as strings, etc. Defeats the point of an Excel export.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Click any column header in Day Book -&gt; nothing happens.</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>1.0.11</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>f3e433d</t>
-        </is>
-      </c>
+          <t>Export Day Book / Trial Balance to Excel -&gt; open in Excel -&gt; try to SUM the Amount column or apply a Date filter -&gt; doesn't work.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr"/>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>New ui/table_utils.py with make_sortable + populating() context manager.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>All tables (amount cols)</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Amount columns sorted lexically -- Rs.10 ranked before Rs.2 because Qt compares cell text as strings.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Sort by Amount on Day Book -- order is wrong.</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>1.0.11</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>f3e433d</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>NumericTableItem stashes raw float in UserRole sort key; __lt__ uses it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>B5</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Internal</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Build pipeline (Nuitka)</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Windows Defender real-time scan locked the freshly-built AccGenie.exe before Nuitka's rcedit step could inject resources. 'Failed to add resources... attempt 5/5, FATAL.' Build aborted.</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Run build/build.bat -&gt; Nuitka completes C-link -&gt; fails on resource injection.</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>1.0.11</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>a08887f</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>Dropped --product-name/version/file-version/file-description/copyright. Version still in installer filename + Inno wizard.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Internal</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Reports -- Balance Sheet</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>'Schedule III (coming soon)' disabled item in the BS format dropdown -- user-facing tech debt with no implementation behind it.</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Open Balance Sheet -&gt; Format dropdown shows a greyed entry that does nothing.</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>1.0.12</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>a7f5354</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>Removed the entry. Re-add when a real Companies Act 2013 categorisation mapping ships.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>B7</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Internal</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>All Rs. formatting</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Python's default ',' grouping produced US-style thousands separators on Indian amounts: Rs.1,234,567.89 instead of the correct Rs.12,34,567.89 (lakh grouping).</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Any amount &gt;= Rs.1 lakh on any report renders with US grouping.</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>1.0.12</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>a7f5354</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>New core/i18n.py with format_currency. Wired in reports_page._fmt (~48 sites) + daybook. Remaining hardcoded Rs.{x:,.2f} sites (exporters, voucher_form, bank_reco) still produce default grouping -- cut over file-by-file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>B8</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Internal</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>License Server</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Seat-release cooldown (24h per key) was firing but the operator was never notified -- license-sharing abuse looked invisible.</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Trip the cooldown: deactivate machine A, immediately re-activate on machine B within 24h. Server returns the cooldown error but no email to ops.</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>1.0.12</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>a7f5354</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>Added _maybe_alert_seat_release_abuse() -- best-effort SMTP send to settings.ops_alert_email; debounced once per key per 24h.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>B9</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>UI Polish</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Buttons too large or too small on multiple screens; some button text not visible (contrast / clipping); 'looks ugly on many screens'.</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>User-reported general impression. Specific screens not yet enumerated.</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>Need user to list the specific screens. C1 in pending_work.xlsx.</t>
+          <t>core/exporters.py needs to set cell.value as float/datetime and apply cell.number_format ('#,##0.00' for currency per locale; 'dd-mmm-yyyy' or per locale for dates). PDF exporter can stay string-rendered.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:K11"/>
+  <autoFilter ref="A2:K5"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>

</xml_diff>

<commit_message>
bug_register: add B4 (date picker visibility) + B5 (txn counting wrong)
B4 — Active dates not visible in date picker (SmartDateEdit). Specific
symptom not yet pinned: could be (a) calendar today/selected styling,
(b) input-field text contrast, (c) digits overlapped by spin arrows.

B5 — Transaction counter inconsistent with the rule "count every
transaction at the pricing values programmed on the day of the
transaction." Code map showed only ui/voucher_form.py increments
(single + multi-party post). Bank reco bulk-create, ledger reco
voucher-creation, AI Document Reader bulk posts, edits, and cancels
all bypass the counter. Plus the counter lives in local license.json,
not server-validated, so the "values programmed on that day" rule
needs a pricing-history snapshot before this can be fixed correctly.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bug_register.xlsx
+++ b/docs/bug_register.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -684,8 +684,106 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Date picker (SmartDateEdit)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Active dates are not visible in the date picker.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>User-reported; specific dialog/page not yet pinned down. Likely the calendar dropdown — today / currently-selected date may be unstyled, or the typed date in the input field may be illegible (contrast / overlap with the spin arrows).</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Probably one of: (a) calendar grid doesn't visually mark today / selected date, (b) input-field text contrast against bg_input is too low, (c) something is overlapping the digits. Confirm with screenshot before fixing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Transaction counter / metering</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Transactions are not being counted properly. Every transaction must be counted against usage per the values programmed on the day the transaction was posted.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Per code map (2026-05-19): counter increments only on manual voucher posts in ui/voucher_form.py (entry page + multi-party dialog). Bank reco bulk-create, ledger reco voucher-creation, AI Document Reader bulk posts, and edits/cancels all bypass the counter entirely.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Domain rule: see [[feedback-accgenie-txn-counting-rule]]. Current behaviour snapshot: see [[project-accgenie-txn-counting-state]]. Gaps: (1) bank/ledger reco vouchers unmetered, (2) AI doc-reader posts unmetered, (3) edits do not increment, (4) cancels do not refund, (5) counter lives in license.json local-only (not server-validated). Need decision on each before fix.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K5"/>
+  <autoFilter ref="A2:K7"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>

</xml_diff>

<commit_message>
bug_register: add B6 — license version ignored on version upgrade
Installing a new version changes the product version but the upgrade
ignores the pre-installed license version — prior activation is lost
or mismatched after upgrade. High severity (a paid user can lose
access on a routine update). License code is shared
(core/license_manager.py, used by RWAGenie too) so the fix lands once.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bug_register.xlsx
+++ b/docs/bug_register.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -782,8 +782,57 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Licensing / version upgrade</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Installing a new version changes the product version but ignores the pre-installed license version — the upgrade does not carry the existing license forward / re-validates against the new version and the prior activation is lost or mismatched.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Install over an existing activated install (e.g. 1.0.11 -&gt; 1.0.12, or 0.1.7 -&gt; 0.1.8). After upgrade the app behaves as if the license is for the old version / is no longer recognised.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>License code is shared: core/license_manager.py (AccGenie) is used by RWAGenie too. Likely the activation record is keyed to product version and an upgrade should treat the licence as version-agnostic (or major-version-scoped). Confirm exact symptom + which file persists the activation before fixing. Cross-app — fix once in the shared manager.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K7"/>
+  <autoFilter ref="A2:K8"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>

</xml_diff>

<commit_message>
bug_register: add B7 — large (~700-line) bank statement may drop rows
User-reported preliminary 2026-05-20: small statements reconcile
fine, but on a ~700-line statement some rows may not have been
picked. Details pending. Note to self when investigating: the
conservative auto-match intentionally leaves ambiguous triples
UNMATCHED — confirm rows are genuinely missing, not just unmatched.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bug_register.xlsx
+++ b/docs/bug_register.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -831,8 +831,57 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>High (TBD)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Bank Reconciliation</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>On a large (~700-line) bank statement, the reconciliation may not have picked up some rows — rows possibly missing after a completed import/reconcile. Small statements work fine.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>User-reported, preliminary — full details pending. Reproduce with the 700-line statement.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>DETAILS PENDING from user. Suspect areas: statement parser dropping rows on a large file; a query LIMIT truncating results; or rows mis-bucketed. NOTE: conservative auto-match deliberately SKIPS ambiguous (date,amount,sign) ties — confirm the 'missing' rows are genuinely absent, not just left UNMATCHED by design.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K8"/>
+  <autoFilter ref="A2:K9"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>

</xml_diff>

<commit_message>
bug_register: B8 — ledger reco cannot resume an in-progress statement
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bug_register.xlsx
+++ b/docs/bug_register.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugs'!$A$2:$K$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -880,8 +880,57 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>B8</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Ledger Reconciliation</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Ledger reconciliation cannot resume an in-progress statement. Bank reco has a Resume flow (recent-imports table with a Resume button + auto-prompt when a ledger is picked); ledger reco's imports table only has Delete — an interrupted ledger reconciliation can't be picked up.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Open Ledger Reconciliation, import a statement, leave it part-done, reopen — no way back to it.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Parity gap vs bank reco — not covered by A10's scope. Port bank reco's find_active_statement + _on_resume_statement + the Resume button + auto-prompt. Best fixed as part of A14 (unify the two reco modules).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K9"/>
+  <autoFilter ref="A2:K10"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>

</xml_diff>